<commit_message>
Update game data with latest results
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manue\Dropbox\Desk\Projects\projects_other\project_ti_auswertung\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB1229E-AC53-4957-81A5-B3158DB936FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C92D878-1BD3-47B7-9BAB-2DF930D66438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2160" yWindow="2160" windowWidth="14400" windowHeight="7270" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="results" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="165">
   <si>
     <t>game_id</t>
   </si>
@@ -510,6 +510,27 @@
   </si>
   <si>
     <t>Manu in Aktionsphase 2 VP mit Imperial PO</t>
+  </si>
+  <si>
+    <t>6980d35150cef813bc292d99</t>
+  </si>
+  <si>
+    <t>Frank in Statusphase 2 VP.</t>
+  </si>
+  <si>
+    <t>winner_had_support</t>
+  </si>
+  <si>
+    <t>Konzentriert euch mal</t>
+  </si>
+  <si>
+    <t>Neue Meta: Hauptsache gegen Saar</t>
+  </si>
+  <si>
+    <t>69985ebb02ef39318bb2ed33</t>
+  </si>
+  <si>
+    <t>Eric hatte 9 Punkte; Shard of Throne gefunden. Damit war spiel fertig.</t>
   </si>
 </sst>
 </file>
@@ -835,7 +856,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E127"/>
+  <dimension ref="A1:E135"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.453125" bestFit="1" customWidth="1"/>
@@ -3004,6 +3025,130 @@
         <v>3</v>
       </c>
     </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A128" t="s">
+        <v>158</v>
+      </c>
+      <c r="B128" t="s">
+        <v>9</v>
+      </c>
+      <c r="C128">
+        <v>10</v>
+      </c>
+      <c r="D128" t="s">
+        <v>45</v>
+      </c>
+      <c r="E128">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A129" t="s">
+        <v>158</v>
+      </c>
+      <c r="B129" t="s">
+        <v>15</v>
+      </c>
+      <c r="C129">
+        <v>9</v>
+      </c>
+      <c r="D129" t="s">
+        <v>24</v>
+      </c>
+      <c r="E129">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A130" t="s">
+        <v>158</v>
+      </c>
+      <c r="B130" t="s">
+        <v>11</v>
+      </c>
+      <c r="C130">
+        <v>8</v>
+      </c>
+      <c r="D130" t="s">
+        <v>47</v>
+      </c>
+      <c r="E130">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A131" t="s">
+        <v>158</v>
+      </c>
+      <c r="B131" t="s">
+        <v>50</v>
+      </c>
+      <c r="C131">
+        <v>6</v>
+      </c>
+      <c r="D131" t="s">
+        <v>22</v>
+      </c>
+      <c r="E131">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A132" t="s">
+        <v>163</v>
+      </c>
+      <c r="B132" t="s">
+        <v>11</v>
+      </c>
+      <c r="C132">
+        <v>10</v>
+      </c>
+      <c r="D132" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A133" t="s">
+        <v>163</v>
+      </c>
+      <c r="B133" t="s">
+        <v>9</v>
+      </c>
+      <c r="C133">
+        <v>7</v>
+      </c>
+      <c r="D133" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A134" t="s">
+        <v>163</v>
+      </c>
+      <c r="B134" t="s">
+        <v>50</v>
+      </c>
+      <c r="C134">
+        <v>6</v>
+      </c>
+      <c r="D134" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A135" t="s">
+        <v>163</v>
+      </c>
+      <c r="B135" t="s">
+        <v>15</v>
+      </c>
+      <c r="C135">
+        <v>5</v>
+      </c>
+      <c r="D135" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3012,17 +3157,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B8F1982-CDD4-4795-9923-90E8136A1DF7}">
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.81640625" customWidth="1"/>
     <col min="2" max="2" width="25.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="10.90625" style="1"/>
-    <col min="7" max="7" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.1796875" hidden="1" customWidth="1"/>
+    <col min="4" max="5" width="0" style="1" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="0" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="11.90625" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="18.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3045,10 +3192,13 @@
         <v>121</v>
       </c>
       <c r="H1" t="s">
+        <v>160</v>
+      </c>
+      <c r="I1" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -3070,11 +3220,14 @@
       <c r="G2" t="s">
         <v>122</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>48</v>
       </c>
@@ -3096,11 +3249,14 @@
       <c r="G3" t="s">
         <v>122</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>51</v>
       </c>
@@ -3122,11 +3278,14 @@
       <c r="G4" t="s">
         <v>124</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>53</v>
       </c>
@@ -3148,11 +3307,14 @@
       <c r="G5" t="s">
         <v>124</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>55</v>
       </c>
@@ -3174,11 +3336,14 @@
       <c r="G6" t="s">
         <v>125</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>57</v>
       </c>
@@ -3200,11 +3365,14 @@
       <c r="G7" t="s">
         <v>124</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>59</v>
       </c>
@@ -3226,11 +3394,14 @@
       <c r="G8" t="s">
         <v>122</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>61</v>
       </c>
@@ -3252,11 +3423,14 @@
       <c r="G9" t="s">
         <v>122</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>64</v>
       </c>
@@ -3278,11 +3452,14 @@
       <c r="G10" t="s">
         <v>124</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>66</v>
       </c>
@@ -3304,11 +3481,14 @@
       <c r="G11" t="s">
         <v>122</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>68</v>
       </c>
@@ -3330,11 +3510,14 @@
       <c r="G12" t="s">
         <v>125</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>70</v>
       </c>
@@ -3356,11 +3539,14 @@
       <c r="G13" t="s">
         <v>124</v>
       </c>
-      <c r="H13" t="s">
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>72</v>
       </c>
@@ -3382,11 +3568,14 @@
       <c r="G14" t="s">
         <v>124</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>74</v>
       </c>
@@ -3408,11 +3597,14 @@
       <c r="G15" t="s">
         <v>122</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H15">
+        <v>1</v>
+      </c>
+      <c r="I15" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>76</v>
       </c>
@@ -3434,11 +3626,14 @@
       <c r="G16" t="s">
         <v>122</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>78</v>
       </c>
@@ -3460,11 +3655,14 @@
       <c r="G17" t="s">
         <v>122</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H17">
+        <v>0</v>
+      </c>
+      <c r="I17" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>80</v>
       </c>
@@ -3486,11 +3684,14 @@
       <c r="G18" t="s">
         <v>124</v>
       </c>
-      <c r="H18" t="s">
+      <c r="H18">
+        <v>1</v>
+      </c>
+      <c r="I18" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>82</v>
       </c>
@@ -3512,11 +3713,14 @@
       <c r="G19" t="s">
         <v>122</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>83</v>
       </c>
@@ -3538,11 +3742,14 @@
       <c r="G20" t="s">
         <v>124</v>
       </c>
-      <c r="H20" t="s">
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>85</v>
       </c>
@@ -3564,11 +3771,11 @@
       <c r="G21" t="s">
         <v>122</v>
       </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>87</v>
       </c>
@@ -3590,11 +3797,11 @@
       <c r="G22" t="s">
         <v>122</v>
       </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>89</v>
       </c>
@@ -3616,11 +3823,11 @@
       <c r="G23" t="s">
         <v>124</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>91</v>
       </c>
@@ -3642,11 +3849,11 @@
       <c r="G24" t="s">
         <v>124</v>
       </c>
-      <c r="H24" t="s">
+      <c r="I24" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>93</v>
       </c>
@@ -3668,11 +3875,11 @@
       <c r="G25" t="s">
         <v>124</v>
       </c>
-      <c r="H25" t="s">
+      <c r="I25" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>94</v>
       </c>
@@ -3694,11 +3901,11 @@
       <c r="G26" t="s">
         <v>125</v>
       </c>
-      <c r="H26" t="s">
+      <c r="I26" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>96</v>
       </c>
@@ -3720,11 +3927,11 @@
       <c r="G27" t="s">
         <v>124</v>
       </c>
-      <c r="H27" t="s">
+      <c r="I27" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>100</v>
       </c>
@@ -3746,11 +3953,11 @@
       <c r="G28" t="s">
         <v>122</v>
       </c>
-      <c r="H28" t="s">
+      <c r="I28" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>102</v>
       </c>
@@ -3772,11 +3979,11 @@
       <c r="G29" t="s">
         <v>122</v>
       </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>104</v>
       </c>
@@ -3798,11 +4005,11 @@
       <c r="G30" t="s">
         <v>122</v>
       </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>107</v>
       </c>
@@ -3824,11 +4031,11 @@
       <c r="G31" t="s">
         <v>124</v>
       </c>
-      <c r="H31" t="s">
+      <c r="I31" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>109</v>
       </c>
@@ -3850,11 +4057,11 @@
       <c r="G32" t="s">
         <v>122</v>
       </c>
-      <c r="H32" t="s">
+      <c r="I32" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>110</v>
       </c>
@@ -3876,11 +4083,11 @@
       <c r="G33" t="s">
         <v>122</v>
       </c>
-      <c r="H33" t="s">
+      <c r="I33" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>112</v>
       </c>
@@ -3902,11 +4109,11 @@
       <c r="G34" t="s">
         <v>124</v>
       </c>
-      <c r="H34" t="s">
+      <c r="I34" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>113</v>
       </c>
@@ -3928,11 +4135,11 @@
       <c r="G35" t="s">
         <v>122</v>
       </c>
-      <c r="H35" t="s">
+      <c r="I35" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>114</v>
       </c>
@@ -3954,11 +4161,11 @@
       <c r="G36" t="s">
         <v>124</v>
       </c>
-      <c r="H36" t="s">
+      <c r="I36" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>115</v>
       </c>
@@ -3980,8 +4187,66 @@
       <c r="G37" t="s">
         <v>124</v>
       </c>
-      <c r="H37" t="s">
+      <c r="I37" t="s">
         <v>157</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>158</v>
+      </c>
+      <c r="B38" t="s">
+        <v>161</v>
+      </c>
+      <c r="C38">
+        <v>10</v>
+      </c>
+      <c r="D38" s="1">
+        <v>46055</v>
+      </c>
+      <c r="E38" s="1">
+        <v>46073</v>
+      </c>
+      <c r="F38">
+        <v>5</v>
+      </c>
+      <c r="G38" t="s">
+        <v>122</v>
+      </c>
+      <c r="H38">
+        <v>1</v>
+      </c>
+      <c r="I38" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>163</v>
+      </c>
+      <c r="B39" t="s">
+        <v>162</v>
+      </c>
+      <c r="C39">
+        <v>10</v>
+      </c>
+      <c r="D39" s="1">
+        <v>46073</v>
+      </c>
+      <c r="E39" s="1">
+        <v>46091</v>
+      </c>
+      <c r="F39">
+        <v>5</v>
+      </c>
+      <c r="G39" t="s">
+        <v>124</v>
+      </c>
+      <c r="H39">
+        <v>1</v>
+      </c>
+      <c r="I39" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add game results for Brave Manus Mom (game 69d64abae5d942b95680c51e)
Manu (Saar) wins 10 VP via Agendaphase with Imperial + open 1VP PO.
Thomas (Xxcha) 5 VP, Eric (Mentak) 5 VP. Updated ti_data.json via pipeline.

https://claude.ai/code/session_01Gnv2Z33Z6VLcTtYb4Sp1TX
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -19,8 +19,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -51,8 +51,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -419,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,10 +485,10 @@
       <c r="C2" t="n">
         <v>10</v>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D2" s="2" t="n">
         <v>45072</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="2" t="n">
         <v>45120</v>
       </c>
       <c r="F2" t="n">
@@ -520,10 +522,10 @@
       <c r="C3" t="n">
         <v>10</v>
       </c>
-      <c r="D3" s="1" t="n">
+      <c r="D3" s="2" t="n">
         <v>45114</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>45135</v>
       </c>
       <c r="F3" t="n">
@@ -557,10 +559,10 @@
       <c r="C4" t="n">
         <v>10</v>
       </c>
-      <c r="D4" s="1" t="n">
+      <c r="D4" s="2" t="n">
         <v>45137</v>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="2" t="n">
         <v>45151</v>
       </c>
       <c r="F4" t="n">
@@ -594,10 +596,10 @@
       <c r="C5" t="n">
         <v>14</v>
       </c>
-      <c r="D5" s="1" t="n">
+      <c r="D5" s="2" t="n">
         <v>45182</v>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="2" t="n">
         <v>45211</v>
       </c>
       <c r="F5" t="n">
@@ -631,10 +633,10 @@
       <c r="C6" t="n">
         <v>14</v>
       </c>
-      <c r="D6" s="1" t="n">
+      <c r="D6" s="2" t="n">
         <v>45212</v>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="E6" s="2" t="n">
         <v>45239</v>
       </c>
       <c r="F6" t="n">
@@ -668,10 +670,10 @@
       <c r="C7" t="n">
         <v>14</v>
       </c>
-      <c r="D7" s="1" t="n">
+      <c r="D7" s="2" t="n">
         <v>45301</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>45331</v>
       </c>
       <c r="F7" t="n">
@@ -705,10 +707,10 @@
       <c r="C8" t="n">
         <v>14</v>
       </c>
-      <c r="D8" s="1" t="n">
+      <c r="D8" s="2" t="n">
         <v>45334</v>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>45366</v>
       </c>
       <c r="F8" t="n">
@@ -742,10 +744,10 @@
       <c r="C9" t="n">
         <v>14</v>
       </c>
-      <c r="D9" s="1" t="n">
+      <c r="D9" s="2" t="n">
         <v>45367</v>
       </c>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="2" t="n">
         <v>45384</v>
       </c>
       <c r="F9" t="n">
@@ -779,10 +781,10 @@
       <c r="C10" t="n">
         <v>14</v>
       </c>
-      <c r="D10" s="1" t="n">
+      <c r="D10" s="2" t="n">
         <v>45385</v>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="2" t="n">
         <v>45395</v>
       </c>
       <c r="F10" t="n">
@@ -816,10 +818,10 @@
       <c r="C11" t="n">
         <v>14</v>
       </c>
-      <c r="D11" s="1" t="n">
+      <c r="D11" s="2" t="n">
         <v>45395</v>
       </c>
-      <c r="E11" s="1" t="n">
+      <c r="E11" s="2" t="n">
         <v>45419</v>
       </c>
       <c r="F11" t="n">
@@ -853,10 +855,10 @@
       <c r="C12" t="n">
         <v>14</v>
       </c>
-      <c r="D12" s="1" t="n">
+      <c r="D12" s="2" t="n">
         <v>45473</v>
       </c>
-      <c r="E12" s="1" t="n">
+      <c r="E12" s="2" t="n">
         <v>45506</v>
       </c>
       <c r="F12" t="n">
@@ -890,10 +892,10 @@
       <c r="C13" t="n">
         <v>10</v>
       </c>
-      <c r="D13" s="1" t="n">
+      <c r="D13" s="2" t="n">
         <v>45516</v>
       </c>
-      <c r="E13" s="1" t="n">
+      <c r="E13" s="2" t="n">
         <v>45528</v>
       </c>
       <c r="F13" t="n">
@@ -927,10 +929,10 @@
       <c r="C14" t="n">
         <v>10</v>
       </c>
-      <c r="D14" s="1" t="n">
+      <c r="D14" s="2" t="n">
         <v>45529</v>
       </c>
-      <c r="E14" s="1" t="n">
+      <c r="E14" s="2" t="n">
         <v>45558</v>
       </c>
       <c r="F14" t="n">
@@ -964,10 +966,10 @@
       <c r="C15" t="n">
         <v>10</v>
       </c>
-      <c r="D15" s="1" t="n">
+      <c r="D15" s="2" t="n">
         <v>45559</v>
       </c>
-      <c r="E15" s="1" t="n">
+      <c r="E15" s="2" t="n">
         <v>45574</v>
       </c>
       <c r="F15" t="n">
@@ -1001,10 +1003,10 @@
       <c r="C16" t="n">
         <v>10</v>
       </c>
-      <c r="D16" s="1" t="n">
+      <c r="D16" s="2" t="n">
         <v>45589</v>
       </c>
-      <c r="E16" s="1" t="n">
+      <c r="E16" s="2" t="n">
         <v>45613</v>
       </c>
       <c r="F16" t="n">
@@ -1038,10 +1040,10 @@
       <c r="C17" t="n">
         <v>14</v>
       </c>
-      <c r="D17" s="1" t="n">
+      <c r="D17" s="2" t="n">
         <v>45700</v>
       </c>
-      <c r="E17" s="1" t="n">
+      <c r="E17" s="2" t="n">
         <v>45735</v>
       </c>
       <c r="F17" t="n">
@@ -1075,10 +1077,10 @@
       <c r="C18" t="n">
         <v>10</v>
       </c>
-      <c r="D18" s="1" t="n">
+      <c r="D18" s="2" t="n">
         <v>45735</v>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="2" t="n">
         <v>45749</v>
       </c>
       <c r="F18" t="n">
@@ -1112,10 +1114,10 @@
       <c r="C19" t="n">
         <v>10</v>
       </c>
-      <c r="D19" s="1" t="n">
+      <c r="D19" s="2" t="n">
         <v>45750</v>
       </c>
-      <c r="E19" s="1" t="n">
+      <c r="E19" s="2" t="n">
         <v>45756</v>
       </c>
       <c r="F19" t="n">
@@ -1149,10 +1151,10 @@
       <c r="C20" t="n">
         <v>10</v>
       </c>
-      <c r="D20" s="1" t="n">
+      <c r="D20" s="2" t="n">
         <v>45756</v>
       </c>
-      <c r="E20" s="1" t="n">
+      <c r="E20" s="2" t="n">
         <v>45764</v>
       </c>
       <c r="F20" t="n">
@@ -1186,10 +1188,10 @@
       <c r="C21" t="n">
         <v>10</v>
       </c>
-      <c r="D21" s="1" t="n">
+      <c r="D21" s="2" t="n">
         <v>45765</v>
       </c>
-      <c r="E21" s="1" t="n">
+      <c r="E21" s="2" t="n">
         <v>45783</v>
       </c>
       <c r="F21" t="n">
@@ -1200,7 +1202,6 @@
           <t>Statusphase</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>Thomas in Statusphase 1 VP mit PO</t>
@@ -1221,10 +1222,10 @@
       <c r="C22" t="n">
         <v>10</v>
       </c>
-      <c r="D22" s="1" t="n">
+      <c r="D22" s="2" t="n">
         <v>45785</v>
       </c>
-      <c r="E22" s="1" t="n">
+      <c r="E22" s="2" t="n">
         <v>45796</v>
       </c>
       <c r="F22" t="n">
@@ -1235,7 +1236,6 @@
           <t>Statusphase</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>Manu in Statusphase, 1 VP mit PO</t>
@@ -1256,10 +1256,10 @@
       <c r="C23" t="n">
         <v>10</v>
       </c>
-      <c r="D23" s="1" t="n">
+      <c r="D23" s="2" t="n">
         <v>45809</v>
       </c>
-      <c r="E23" s="1" t="n">
+      <c r="E23" s="2" t="n">
         <v>45826</v>
       </c>
       <c r="F23" t="n">
@@ -1270,7 +1270,6 @@
           <t>Aktionsphase</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>Manu in Aktionsphase mit Imperial 1 VP PO</t>
@@ -1291,10 +1290,10 @@
       <c r="C24" t="n">
         <v>10</v>
       </c>
-      <c r="D24" s="1" t="n">
+      <c r="D24" s="2" t="n">
         <v>45817</v>
       </c>
-      <c r="E24" s="1" t="n">
+      <c r="E24" s="2" t="n">
         <v>45832</v>
       </c>
       <c r="F24" t="n">
@@ -1305,7 +1304,6 @@
           <t>Aktionsphase</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>Thomas in Aktionsphase mit Sekret Destroy Their greates Ship</t>
@@ -1326,10 +1324,10 @@
       <c r="C25" t="n">
         <v>10</v>
       </c>
-      <c r="D25" s="1" t="n">
+      <c r="D25" s="2" t="n">
         <v>45832</v>
       </c>
-      <c r="E25" s="1" t="n">
+      <c r="E25" s="2" t="n">
         <v>45856</v>
       </c>
       <c r="F25" t="n">
@@ -1340,7 +1338,6 @@
           <t>Aktionsphase</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>Eric in Aktionsphase durch Shard of the Throne</t>
@@ -1361,10 +1358,10 @@
       <c r="C26" t="n">
         <v>10</v>
       </c>
-      <c r="D26" s="1" t="n">
+      <c r="D26" s="2" t="n">
         <v>45856</v>
       </c>
-      <c r="E26" s="1" t="n">
+      <c r="E26" s="2" t="n">
         <v>45861</v>
       </c>
       <c r="F26" t="n">
@@ -1375,7 +1372,6 @@
           <t>Agendaphase</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>Eric in Agendaphase durch Mutiny</t>
@@ -1396,10 +1392,10 @@
       <c r="C27" t="n">
         <v>10</v>
       </c>
-      <c r="D27" s="1" t="n">
+      <c r="D27" s="2" t="n">
         <v>45861</v>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="E27" s="2" t="n">
         <v>45868</v>
       </c>
       <c r="F27" t="n">
@@ -1410,7 +1406,6 @@
           <t>Aktionsphase</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
           <t>Manu in Aktionsphase durch Spark a Rebellion</t>
@@ -1431,10 +1426,10 @@
       <c r="C28" t="n">
         <v>10</v>
       </c>
-      <c r="D28" s="1" t="n">
+      <c r="D28" s="2" t="n">
         <v>45868</v>
       </c>
-      <c r="E28" s="1" t="n">
+      <c r="E28" s="2" t="n">
         <v>45873</v>
       </c>
       <c r="F28" t="n">
@@ -1445,7 +1440,6 @@
           <t>Statusphase</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>Thomas in Statusphase 2 VP, 1 PO 1 Sekret</t>
@@ -1466,10 +1460,10 @@
       <c r="C29" t="n">
         <v>10</v>
       </c>
-      <c r="D29" s="1" t="n">
+      <c r="D29" s="2" t="n">
         <v>45873</v>
       </c>
-      <c r="E29" s="1" t="n">
+      <c r="E29" s="2" t="n">
         <v>45882</v>
       </c>
       <c r="F29" t="n">
@@ -1480,7 +1474,6 @@
           <t>Statusphase</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>Thomas in Statusphase 2 VP durch PO</t>
@@ -1501,10 +1494,10 @@
       <c r="C30" t="n">
         <v>10</v>
       </c>
-      <c r="D30" s="1" t="n">
+      <c r="D30" s="2" t="n">
         <v>45882</v>
       </c>
-      <c r="E30" s="1" t="n">
+      <c r="E30" s="2" t="n">
         <v>45892</v>
       </c>
       <c r="F30" t="n">
@@ -1515,7 +1508,6 @@
           <t>Statusphase</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>Eric in Statusphase mit 3VP, 2 PO und 1 Sekret</t>
@@ -1536,10 +1528,10 @@
       <c r="C31" t="n">
         <v>10</v>
       </c>
-      <c r="D31" s="1" t="n">
+      <c r="D31" s="2" t="n">
         <v>45892</v>
       </c>
-      <c r="E31" s="1" t="n">
+      <c r="E31" s="2" t="n">
         <v>45897</v>
       </c>
       <c r="F31" t="n">
@@ -1550,7 +1542,6 @@
           <t>Aktionsphase</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>Eric in Aktionsphase, Demonstrate your Power</t>
@@ -1571,10 +1562,10 @@
       <c r="C32" t="n">
         <v>10</v>
       </c>
-      <c r="D32" s="1" t="n">
+      <c r="D32" s="2" t="n">
         <v>45898</v>
       </c>
-      <c r="E32" s="1" t="n">
+      <c r="E32" s="2" t="n">
         <v>45915</v>
       </c>
       <c r="F32" t="n">
@@ -1585,7 +1576,6 @@
           <t>Statusphase</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>Eric in Statusphase 2 VP, 1 PO und 1 Sekret</t>
@@ -1606,10 +1596,10 @@
       <c r="C33" t="n">
         <v>10</v>
       </c>
-      <c r="D33" s="1" t="n">
+      <c r="D33" s="2" t="n">
         <v>45915</v>
       </c>
-      <c r="E33" s="1" t="n">
+      <c r="E33" s="2" t="n">
         <v>45959</v>
       </c>
       <c r="F33" t="n">
@@ -1620,7 +1610,6 @@
           <t>Statusphase</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>Manu in Statusphase, 1 VP mit PO</t>
@@ -1641,10 +1630,10 @@
       <c r="C34" t="n">
         <v>10</v>
       </c>
-      <c r="D34" s="1" t="n">
+      <c r="D34" s="2" t="n">
         <v>46006</v>
       </c>
-      <c r="E34" s="1" t="n">
+      <c r="E34" s="2" t="n">
         <v>46018</v>
       </c>
       <c r="F34" t="n">
@@ -1655,7 +1644,6 @@
           <t>Aktionsphase</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
           <t>Thomas in Aktionsphase mit Imperial und 2 VP PO</t>
@@ -1676,10 +1664,10 @@
       <c r="C35" t="n">
         <v>10</v>
       </c>
-      <c r="D35" s="1" t="n">
+      <c r="D35" s="2" t="n">
         <v>46018</v>
       </c>
-      <c r="E35" s="1" t="n">
+      <c r="E35" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="F35" t="n">
@@ -1690,7 +1678,6 @@
           <t>Statusphase</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>Eric in Statusphase 2 VP, 1 PO und 1 Sekret</t>
@@ -1711,10 +1698,10 @@
       <c r="C36" t="n">
         <v>10</v>
       </c>
-      <c r="D36" s="1" t="n">
+      <c r="D36" s="2" t="n">
         <v>46032</v>
       </c>
-      <c r="E36" s="1" t="n">
+      <c r="E36" s="2" t="n">
         <v>46037</v>
       </c>
       <c r="F36" t="n">
@@ -1725,7 +1712,6 @@
           <t>Aktionsphase</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
           <t>Thomas in Aktionsphase 1 VP mit Imperial MR</t>
@@ -1746,10 +1732,10 @@
       <c r="C37" t="n">
         <v>10</v>
       </c>
-      <c r="D37" s="1" t="n">
+      <c r="D37" s="2" t="n">
         <v>46040</v>
       </c>
-      <c r="E37" s="1" t="n">
+      <c r="E37" s="2" t="n">
         <v>46055</v>
       </c>
       <c r="F37" t="n">
@@ -1760,7 +1746,6 @@
           <t>Aktionsphase</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>Manu in Aktionsphase 2 VP mit Imperial PO</t>
@@ -1781,10 +1766,10 @@
       <c r="C38" t="n">
         <v>10</v>
       </c>
-      <c r="D38" s="1" t="n">
+      <c r="D38" s="2" t="n">
         <v>46055</v>
       </c>
-      <c r="E38" s="1" t="n">
+      <c r="E38" s="2" t="n">
         <v>46073</v>
       </c>
       <c r="F38" t="n">
@@ -1818,10 +1803,10 @@
       <c r="C39" t="n">
         <v>10</v>
       </c>
-      <c r="D39" s="1" t="n">
+      <c r="D39" s="2" t="n">
         <v>46073</v>
       </c>
-      <c r="E39" s="1" t="n">
+      <c r="E39" s="2" t="n">
         <v>46091</v>
       </c>
       <c r="F39" t="n">
@@ -1855,10 +1840,10 @@
       <c r="C40" t="n">
         <v>10</v>
       </c>
-      <c r="D40" s="1" t="n">
+      <c r="D40" s="2" t="n">
         <v>46111</v>
       </c>
-      <c r="E40" s="1" t="n">
+      <c r="E40" s="2" t="n">
         <v>46120</v>
       </c>
       <c r="F40" t="n">
@@ -1872,7 +1857,43 @@
       <c r="H40" t="n">
         <v>0</v>
       </c>
-      <c r="I40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>69d64abae5d942b95680c51e</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Brave Manus Mom</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>10</v>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>46120</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>46124</v>
+      </c>
+      <c r="F41" t="n">
+        <v>5</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Agendaphase</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Manu hatte imperial und ein noch ein offenes 1er PO</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1885,7 +1906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E138"/>
+  <dimension ref="A1:E141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4924,7 +4945,6 @@
           <t>Sol</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4945,7 +4965,6 @@
           <t>Barony</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4966,7 +4985,6 @@
           <t>Mentak</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4987,7 +5005,6 @@
           <t>Creuss</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -5008,7 +5025,6 @@
           <t>Naalu</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -5029,7 +5045,6 @@
           <t>L1Z1X</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -5050,7 +5065,75 @@
           <t>Barony</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>69d64abae5d942b95680c51e</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Manu</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>10</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Saar</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>69d64abae5d942b95680c51e</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>5</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Xxcha</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>69d64abae5d942b95680c51e</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Eric</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>5</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Mentak</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add game data: Straffällige Hopfenzupfer (42 games total)
Fixes update_ti_stats.py bug that wiped previous games; restores full 41-game
history and adds the new game correctly.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -17,9 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -50,11 +51,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -420,18 +422,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="25.453125" customWidth="1" min="2" max="2"/>
-    <col width="28.1796875" customWidth="1" min="3" max="3"/>
-    <col width="22.81640625" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="17.7265625" bestFit="1" customWidth="1" min="5" max="6"/>
-    <col width="6.7265625" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="12.08984375" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="18.453125" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="119.453125" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="28.1796875" customWidth="1" min="2" max="2"/>
+    <col width="22.81640625" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="17.7265625" bestFit="1" customWidth="1" min="4" max="5"/>
+    <col width="6.7265625" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="12.08984375" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="18.453125" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="119.453125" bestFit="1" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -442,258 +443,1722 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>game_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>game_max_victory_points</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>start_date</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>rounds</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>win_category</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>winner_had_support</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>win_description</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>game_medium</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>game_name</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>game_max_victory_points</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>start_date</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>end_date</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>rounds</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>win_category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>winner_had_support</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>win_description</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>6470772d0cc21e00141af1a5</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bier aus dem Schlauch trinken</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>45072</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>45120</v>
+      </c>
+      <c r="F2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Statusphase, Starki Naalu 3 VP mit Public und Sekret</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>64a81dbdee77a100148764db</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Becher aus dem Eimer trinken</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>45114</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>45135</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Statusphase, Manu Jol 2 VP mit 1 Public und Sekret, hatte auch Imperial aber nur für 1 PO (nicht MR) in Runde. Speaker letzte Runde war Eric </t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>64c613eaff62200014307719</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Wasser-Schlauch</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>45137</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>45151</v>
+      </c>
+      <c r="F4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Aktionsphase: Manu spielt Imperial und scort Lead from the Front</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>64d90d6450dd3a00140001a4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>14 p Smackup PoK</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>45182</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>45211</v>
+      </c>
+      <c r="F5" t="n">
+        <v>7</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Eric in Aktionphase, hatte auch Imperial für 2 VP PO, Sieg aber unklar warum</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>65299e47784ff00014f0c41e</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Wer hat hier die Hosen unten?</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>45212</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>45239</v>
+      </c>
+      <c r="F6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Agendaphase</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Win in Agendaphase, da Political Censure</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>659e96e2ac9f8b0014b3bebe</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Friedliches verprügeln</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>14</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>45301</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>45331</v>
+      </c>
+      <c r="F7" t="n">
+        <v>8</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Sieg Eric in Aktionphase durch Sekret Destroy Their greatest ship</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>65ca2a4db77b720015197bfc</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Wollen wir Freunde sein?</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>14</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>45334</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>45366</v>
+      </c>
+      <c r="F8" t="n">
+        <v>7</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Thomas in Statusphase 2 VP, 1 PO 1 Sekret</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>65f53e0342cb1900153c80c5</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Flotter Dreier</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>14</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>45367</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>45384</v>
+      </c>
+      <c r="F9" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Thomas in Statusphase 2 VP mit PO</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>660d18b4c063f10015c5cc1b</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Flotter Dreier 2</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>45385</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>45395</v>
+      </c>
+      <c r="F10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Manu in Aktionsphase mit Imperial 1 VP PO</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>661ab137778a0700151551b1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Flotter Vierer</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>14</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>45395</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>45419</v>
+      </c>
+      <c r="F11" t="n">
+        <v>6</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Eric in Statusphase mit 2VP PO</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>6681c55edcefb80015097c5e</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Exploration 4 the win</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>14</v>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>45473</v>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>45506</v>
+      </c>
+      <c r="F12" t="n">
+        <v>6</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Agendaphase</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Eric in Agendaphase mit Crown of Emphidia</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>66ba6de1bb6d9e0015cc8d78</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Shizzle</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>45516</v>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>45528</v>
+      </c>
+      <c r="F13" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Frank, Aktionsphase, Sekret Destroy their greatest Ship</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>66cb1f970823e40015140021</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>5er shizzle</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>45529</v>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>45558</v>
+      </c>
+      <c r="F14" t="n">
+        <v>7</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Manu, Aktionsphase, Sekret Destroy their greatest Ship</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>66f25b8501afda00150d7336</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Langweilig</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>45559</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>45574</v>
+      </c>
+      <c r="F15" t="n">
+        <v>5</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Eric, Statusphase 1 VP mit Sekret</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>671a3e89a022f1de55f3a8bf</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Manu trösten</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>10</v>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>45589</v>
+      </c>
+      <c r="E16" s="1" t="n">
+        <v>45613</v>
+      </c>
+      <c r="F16" t="n">
+        <v>5</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Frank, Statusphase 1 VP mit PO</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>67ac6dfb12236650d4f0cfdc</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Viehrer</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>14</v>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>45700</v>
+      </c>
+      <c r="E17" s="1" t="n">
+        <v>45735</v>
+      </c>
+      <c r="F17" t="n">
+        <v>8</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Thomas, Statusphase, 1 VP mit PO</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>67da6966babd5a850a447f42</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Ficken</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>45735</v>
+      </c>
+      <c r="E18" s="1" t="n">
+        <v>45749</v>
+      </c>
+      <c r="F18" t="n">
+        <v>5</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Thomas durch Support Trade</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>67ee493d7c52833bd9a020fb</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Flotter Dreier</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>10</v>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>45750</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>45756</v>
+      </c>
+      <c r="F19" t="n">
+        <v>6</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Manu in Statusphase, 2 VP mit PO</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>67f6ca41c550f0ebca2e75d8</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Ficki ficki</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>10</v>
+      </c>
+      <c r="D20" s="1" t="n">
+        <v>45756</v>
+      </c>
+      <c r="E20" s="1" t="n">
+        <v>45764</v>
+      </c>
+      <c r="F20" t="n">
+        <v>6</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Eric in Aktionsphase mit Imperial, 1 VP PO und 1 VP MR</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>68026115a5dd682b58b16a39</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Brave and Stupid</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>45765</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>45783</v>
+      </c>
+      <c r="F21" t="n">
+        <v>5</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Thomas in Statusphase 1 VP mit PO</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>681c7d10d5e12c112a6445d8</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>L1 went awol</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>10</v>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>45785</v>
+      </c>
+      <c r="E22" s="1" t="n">
+        <v>45796</v>
+      </c>
+      <c r="F22" t="n">
+        <v>5</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Manu in Statusphase, 1 VP mit PO</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>683c3f4c96bda541c8e1a373</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>MW-Verlängerung</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>45809</v>
+      </c>
+      <c r="E23" s="1" t="n">
+        <v>45826</v>
+      </c>
+      <c r="F23" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Manu in Aktionsphase mit Imperial 1 VP PO</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>6846eff205247103cf2f6010</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Flotter Dreier</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>10</v>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>45817</v>
+      </c>
+      <c r="E24" s="1" t="n">
+        <v>45832</v>
+      </c>
+      <c r="F24" t="n">
+        <v>7</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Thomas in Aktionsphase mit Sekret Destroy Their greates Ship</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>685a87538030b9b281c0cc33</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0 Rage erlaubt, kein sftt swap</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>10</v>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>45832</v>
+      </c>
+      <c r="E25" s="1" t="n">
+        <v>45856</v>
+      </c>
+      <c r="F25" t="n">
+        <v>6</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Eric in Aktionsphase durch Shard of the Throne</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>687a6a4081785bc35b20802f</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Zutiefst Zuwieder wieder</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>10</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>45856</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>45861</v>
+      </c>
+      <c r="F26" t="n">
+        <v>5</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Agendaphase</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Eric in Agendaphase durch Mutiny</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>68809ebcbfbc93cec5b50d0d</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Zutiefst Zuwieder wieder</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>10</v>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>45861</v>
+      </c>
+      <c r="E27" s="1" t="n">
+        <v>45868</v>
+      </c>
+      <c r="F27" t="n">
+        <v>6</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Manu in Aktionsphase durch Spark a Rebellion</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>688a7dd06ca999f50a131e99</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Wieder zuwider</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>10</v>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>45868</v>
+      </c>
+      <c r="E28" s="1" t="n">
+        <v>45873</v>
+      </c>
+      <c r="F28" t="n">
+        <v>5</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Thomas in Statusphase 2 VP, 1 PO 1 Sekret</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>6890d53480917d9ada584d8e</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Warten auf mehr PoK Content</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>10</v>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>45873</v>
+      </c>
+      <c r="E29" s="1" t="n">
+        <v>45882</v>
+      </c>
+      <c r="F29" t="n">
+        <v>5</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Thomas in Statusphase 2 VP durch PO</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>689c4340918b578ec61e122e</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Urlaubstimmy</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>10</v>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>45882</v>
+      </c>
+      <c r="E30" s="1" t="n">
+        <v>45892</v>
+      </c>
+      <c r="F30" t="n">
+        <v>6</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Eric in Statusphase mit 3VP, 2 PO und 1 Sekret</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>68aa0a800810ff3ac2687f4e</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Wer hat Manus Mom zuletzt gesehen?</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>10</v>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>45892</v>
+      </c>
+      <c r="E31" s="1" t="n">
+        <v>45897</v>
+      </c>
+      <c r="F31" t="n">
+        <v>5</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Eric in Aktionsphase, Demonstrate your Power</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>68b13bbc8cf23884545eca76</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Mehr aggro sein dieses Mal</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>10</v>
+      </c>
+      <c r="D32" s="1" t="n">
+        <v>45898</v>
+      </c>
+      <c r="E32" s="1" t="n">
+        <v>45915</v>
+      </c>
+      <c r="F32" t="n">
+        <v>5</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Eric in Statusphase 2 VP, 1 PO und 1 Sekret</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>68c807adb5c98b30851ab64c</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Rise and Shine</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>10</v>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>45915</v>
+      </c>
+      <c r="E33" s="1" t="n">
+        <v>45959</v>
+      </c>
+      <c r="F33" t="n">
+        <v>5</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Manu in Statusphase, 1 VP mit PO</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>694079731cb455091b9a92cb</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>The return of the Timmy</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>10</v>
+      </c>
+      <c r="D34" s="1" t="n">
+        <v>46006</v>
+      </c>
+      <c r="E34" s="1" t="n">
+        <v>46018</v>
+      </c>
+      <c r="F34" t="n">
+        <v>5</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Thomas in Aktionsphase mit Imperial und 2 VP PO</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>69505c9be44f36bfafb98b45</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tommy ist einfach Tommy </t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>10</v>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>46018</v>
+      </c>
+      <c r="E35" s="1" t="n">
+        <v>46032</v>
+      </c>
+      <c r="F35" t="n">
+        <v>5</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Eric in Statusphase 2 VP, 1 PO und 1 Sekret</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>6962727b1e677f7a6f600b1e</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Jetzt mal ohne Fehler bitte</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>10</v>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>46032</v>
+      </c>
+      <c r="E36" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="F36" t="n">
+        <v>6</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Thomas in Aktionsphase 1 VP mit Imperial MR</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>696cdb2972af55390d4e54d5</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>TI We verlängert, wenn ihr euch noch in die Augen schauen könnt</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>10</v>
+      </c>
+      <c r="D37" s="1" t="n">
+        <v>46040</v>
+      </c>
+      <c r="E37" s="1" t="n">
+        <v>46055</v>
+      </c>
+      <c r="F37" t="n">
+        <v>5</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Manu in Aktionsphase 2 VP mit Imperial PO</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>6980d35150cef813bc292d99</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Konzentriert euch mal</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>10</v>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>46055</v>
+      </c>
+      <c r="E38" s="1" t="n">
+        <v>46073</v>
+      </c>
+      <c r="F38" t="n">
+        <v>5</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H38" t="n">
+        <v>1</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Frank in Statusphase 2 VP.</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>69985ebb02ef39318bb2ed33</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Neue Meta: Hauptsache gegen Saar</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>10</v>
+      </c>
+      <c r="D39" s="1" t="n">
+        <v>46073</v>
+      </c>
+      <c r="E39" s="1" t="n">
+        <v>46091</v>
+      </c>
+      <c r="F39" t="n">
+        <v>5</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>1</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Eric hatte 9 Punkte; Shard of Throne gefunden. Damit war spiel fertig.</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>69ca336a5e13fcc25a81f0b6</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Rational aufs Mowl</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>10</v>
+      </c>
+      <c r="D40" s="1" t="n">
+        <v>46111</v>
+      </c>
+      <c r="E40" s="1" t="n">
+        <v>46120</v>
+      </c>
+      <c r="F40" t="n">
+        <v>5</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" t="n">
+        <v/>
+      </c>
+      <c r="J40" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>69d64abae5d942b95680c51e</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Brave Manus Mom</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>10</v>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>46120</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>46124</v>
+      </c>
+      <c r="F41" t="n">
+        <v>5</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Agendaphase</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Manu hatte imperial und ein noch ein offenes 1er PO</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>69dbea2cc9418cc13861e19a</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Wer hat Manu in den Wohnwagen gekackt?</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>10</v>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>46124</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>46133</v>
+      </c>
+      <c r="F42" t="n">
+        <v>5</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="n">
+        <v/>
+      </c>
+      <c r="J42" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>6a2118f02c35b142e42c12b2</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Straffällige Hopfenzupfer</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>10</v>
+      </c>
+      <c r="D43" s="4" t="n">
+        <v>46177</v>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>46185</v>
+      </c>
+      <c r="F43" t="n">
+        <v>6</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>1</v>
+      </c>
+      <c r="J43" t="inlineStr">
         <is>
           <t>online</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Straffällige Hopfenzupfer</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E2" s="1" t="n">
-        <v>46177</v>
-      </c>
-      <c r="F2" s="1" t="n">
-        <v>46185</v>
-      </c>
-      <c r="G2" t="n">
-        <v>6</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Aktionsphase</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="E3" s="1" t="n"/>
-      <c r="F3" s="1" t="n"/>
-    </row>
-    <row r="4">
-      <c r="E4" s="1" t="n"/>
-      <c r="F4" s="1" t="n"/>
-    </row>
-    <row r="5">
-      <c r="E5" s="1" t="n"/>
-      <c r="F5" s="1" t="n"/>
-    </row>
-    <row r="6">
-      <c r="E6" s="1" t="n"/>
-      <c r="F6" s="1" t="n"/>
-    </row>
-    <row r="7">
-      <c r="E7" s="1" t="n"/>
-      <c r="F7" s="1" t="n"/>
-    </row>
-    <row r="8">
-      <c r="E8" s="1" t="n"/>
-      <c r="F8" s="1" t="n"/>
-    </row>
-    <row r="9">
-      <c r="E9" s="1" t="n"/>
-      <c r="F9" s="1" t="n"/>
-    </row>
-    <row r="10">
-      <c r="E10" s="1" t="n"/>
-      <c r="F10" s="1" t="n"/>
-    </row>
-    <row r="11">
-      <c r="E11" s="1" t="n"/>
-      <c r="F11" s="1" t="n"/>
-    </row>
-    <row r="12">
-      <c r="E12" s="1" t="n"/>
-      <c r="F12" s="1" t="n"/>
-    </row>
-    <row r="13">
-      <c r="E13" s="1" t="n"/>
-      <c r="F13" s="1" t="n"/>
-    </row>
-    <row r="14">
-      <c r="E14" s="1" t="n"/>
-      <c r="F14" s="1" t="n"/>
-    </row>
-    <row r="15">
-      <c r="E15" s="1" t="n"/>
-      <c r="F15" s="1" t="n"/>
-    </row>
-    <row r="16">
-      <c r="E16" s="1" t="n"/>
-      <c r="F16" s="1" t="n"/>
-    </row>
-    <row r="17">
-      <c r="E17" s="1" t="n"/>
-      <c r="F17" s="1" t="n"/>
-    </row>
-    <row r="18">
-      <c r="E18" s="1" t="n"/>
-      <c r="F18" s="1" t="n"/>
-    </row>
-    <row r="19">
-      <c r="E19" s="1" t="n"/>
-      <c r="F19" s="1" t="n"/>
-    </row>
-    <row r="20">
-      <c r="E20" s="1" t="n"/>
-      <c r="F20" s="1" t="n"/>
-    </row>
-    <row r="21">
-      <c r="E21" s="1" t="n"/>
-      <c r="F21" s="1" t="n"/>
-    </row>
-    <row r="22">
-      <c r="E22" s="1" t="n"/>
-      <c r="F22" s="1" t="n"/>
-    </row>
-    <row r="23">
-      <c r="E23" s="1" t="n"/>
-      <c r="F23" s="1" t="n"/>
-    </row>
-    <row r="24">
-      <c r="E24" s="1" t="n"/>
-      <c r="F24" s="1" t="n"/>
-    </row>
-    <row r="25">
-      <c r="E25" s="1" t="n"/>
-      <c r="F25" s="1" t="n"/>
-    </row>
-    <row r="26">
-      <c r="E26" s="1" t="n"/>
-      <c r="F26" s="1" t="n"/>
-    </row>
-    <row r="27">
-      <c r="E27" s="1" t="n"/>
-      <c r="F27" s="1" t="n"/>
-    </row>
-    <row r="28">
-      <c r="E28" s="1" t="n"/>
-      <c r="F28" s="1" t="n"/>
-    </row>
-    <row r="29">
-      <c r="E29" s="1" t="n"/>
-      <c r="F29" s="1" t="n"/>
-    </row>
-    <row r="30">
-      <c r="E30" s="1" t="n"/>
-      <c r="F30" s="1" t="n"/>
-    </row>
-    <row r="31">
-      <c r="E31" s="1" t="n"/>
-      <c r="F31" s="1" t="n"/>
-    </row>
-    <row r="32">
-      <c r="E32" s="1" t="n"/>
-      <c r="F32" s="1" t="n"/>
-    </row>
-    <row r="33">
-      <c r="E33" s="1" t="n"/>
-      <c r="F33" s="1" t="n"/>
-    </row>
-    <row r="34">
-      <c r="E34" s="1" t="n"/>
-      <c r="F34" s="1" t="n"/>
-    </row>
-    <row r="35">
-      <c r="E35" s="1" t="n"/>
-      <c r="F35" s="1" t="n"/>
-    </row>
-    <row r="36">
-      <c r="E36" s="1" t="n"/>
-      <c r="F36" s="1" t="n"/>
-    </row>
-    <row r="37">
-      <c r="E37" s="1" t="n"/>
-      <c r="F37" s="1" t="n"/>
-    </row>
-    <row r="38">
-      <c r="E38" s="1" t="n"/>
-      <c r="F38" s="1" t="n"/>
-    </row>
-    <row r="39">
-      <c r="E39" s="1" t="n"/>
-      <c r="F39" s="1" t="n"/>
-    </row>
-    <row r="40">
-      <c r="E40" s="1" t="n"/>
-      <c r="F40" s="1" t="n"/>
-    </row>
-    <row r="41">
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="2" t="n"/>
-    </row>
-    <row r="42">
-      <c r="E42" s="3" t="n"/>
-      <c r="F42" s="3" t="n"/>
-    </row>
-    <row r="43">
-      <c r="E43" s="3" t="n"/>
-      <c r="F43" s="3" t="n"/>
-    </row>
-    <row r="44">
-      <c r="E44" s="3" t="n"/>
-      <c r="F44" s="3" t="n"/>
-    </row>
-    <row r="45">
-      <c r="E45" s="3" t="n"/>
-      <c r="F45" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -706,7 +2171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E153"/>
+  <dimension ref="A1:E147"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3994,7 +5459,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -4017,7 +5482,7 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
@@ -4031,111 +5496,69 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>live0001</t>
-        </is>
+          <t>6a2118f02c35b142e42c12b2</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Eric</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>8</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Empyrean</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>live0001</t>
-        </is>
+          <t>6a2118f02c35b142e42c12b2</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>10</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Sardakk</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>live0001</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>live0001</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>live0002</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>live0003</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
           <t>6a2118f02c35b142e42c12b2</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>Eric</t>
-        </is>
-      </c>
-      <c r="C151" t="n">
-        <v>8</v>
-      </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>Empyrean</t>
-        </is>
-      </c>
-      <c r="E151" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>6a2118f02c35b142e42c12b2</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>Thomas</t>
-        </is>
-      </c>
-      <c r="C152" t="n">
-        <v>10</v>
-      </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>Sardakk</t>
-        </is>
-      </c>
-      <c r="E152" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>6a2118f02c35b142e42c12b2</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
+      <c r="B147" t="inlineStr">
         <is>
           <t>Manu</t>
         </is>
       </c>
-      <c r="C153" t="n">
+      <c r="C147" t="n">
         <v>5</v>
       </c>
-      <c r="D153" t="inlineStr">
+      <c r="D147" t="inlineStr">
         <is>
           <t>Saar</t>
         </is>
       </c>
-      <c r="E153" t="n">
+      <c r="E147" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add game data: Knappheit, des isses
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2154,7 +2154,47 @@
       <c r="H43" t="n">
         <v>1</v>
       </c>
+      <c r="I43" t="n">
+        <v/>
+      </c>
       <c r="J43" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>6a0caa60ac769673103cb9f2</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Knappheit, des isses</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>10</v>
+      </c>
+      <c r="D44" s="4" t="n">
+        <v>46161</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>46175</v>
+      </c>
+      <c r="F44" t="n">
+        <v>5</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>1</v>
+      </c>
+      <c r="J44" t="inlineStr">
         <is>
           <t>online</t>
         </is>
@@ -2171,7 +2211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E147"/>
+  <dimension ref="A1:E150"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5559,6 +5599,75 @@
         </is>
       </c>
       <c r="E147" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>6a0caa60ac769673103cb9f2</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Manu</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>9</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Naalu</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>6a0caa60ac769673103cb9f2</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>7</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Empyrean</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>6a0caa60ac769673103cb9f2</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Eric</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>10</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Yssaril</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add game data: Knappheit, des isses II, Die lustigen 5
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2194,7 +2194,84 @@
       <c r="H44" t="n">
         <v>1</v>
       </c>
+      <c r="I44" t="n">
+        <v/>
+      </c>
       <c r="J44" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>6a2cf93fb2b8d2aa7eb8c3a5</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Knappheit, des isses II</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>10</v>
+      </c>
+      <c r="D45" s="4" t="n">
+        <v>46186</v>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>46193</v>
+      </c>
+      <c r="F45" t="n">
+        <v>5</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>1</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>69256c61fa804c7cd64e3d0f</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Die lustigen 5</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>10</v>
+      </c>
+      <c r="D46" s="4" t="n">
+        <v>45986</v>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>46033</v>
+      </c>
+      <c r="F46" t="n">
+        <v>7</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>1</v>
+      </c>
+      <c r="J46" t="inlineStr">
         <is>
           <t>online</t>
         </is>
@@ -2211,7 +2288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E150"/>
+  <dimension ref="A1:E158"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5669,6 +5746,190 @@
       </c>
       <c r="E150" t="n">
         <v>3</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>6a2cf93fb2b8d2aa7eb8c3a5</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Eric</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>6</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Empyrean</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>6a2cf93fb2b8d2aa7eb8c3a5</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Manu</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>6</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Xxcha</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>6a2cf93fb2b8d2aa7eb8c3a5</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>10</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Saar</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>69256c61fa804c7cd64e3d0f</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Eric</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>6</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>The Yin Brotherhood</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>69256c61fa804c7cd64e3d0f</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Manu</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>10</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Nekro</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>69256c61fa804c7cd64e3d0f</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>alexander.s</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>4</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Empyrean</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>69256c61fa804c7cd64e3d0f</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Lootra</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>4</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Winnu</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>69256c61fa804c7cd64e3d0f</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Michael 🇦🇹</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>3</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Saar</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove 'Die lustigen 5' game (marked irrelevant) and exclude from future syncs
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -2234,6 +2234,9 @@
       <c r="H45" t="n">
         <v>1</v>
       </c>
+      <c r="I45" t="n">
+        <v/>
+      </c>
       <c r="J45" t="inlineStr">
         <is>
           <t>online</t>
@@ -2241,41 +2244,8 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>69256c61fa804c7cd64e3d0f</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Die lustigen 5</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>10</v>
-      </c>
-      <c r="D46" s="4" t="n">
-        <v>45986</v>
-      </c>
-      <c r="E46" s="4" t="n">
-        <v>46033</v>
-      </c>
-      <c r="F46" t="n">
-        <v>7</v>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Statusphase</t>
-        </is>
-      </c>
-      <c r="H46" t="n">
-        <v>1</v>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
+      <c r="D46" s="4" t="n"/>
+      <c r="E46" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5817,121 +5787,11 @@
         <v>3</v>
       </c>
     </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>69256c61fa804c7cd64e3d0f</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>Eric</t>
-        </is>
-      </c>
-      <c r="C154" t="n">
-        <v>6</v>
-      </c>
-      <c r="D154" t="inlineStr">
-        <is>
-          <t>The Yin Brotherhood</t>
-        </is>
-      </c>
-      <c r="E154" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>69256c61fa804c7cd64e3d0f</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>Manu</t>
-        </is>
-      </c>
-      <c r="C155" t="n">
-        <v>10</v>
-      </c>
-      <c r="D155" t="inlineStr">
-        <is>
-          <t>Nekro</t>
-        </is>
-      </c>
-      <c r="E155" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>69256c61fa804c7cd64e3d0f</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>alexander.s</t>
-        </is>
-      </c>
-      <c r="C156" t="n">
-        <v>4</v>
-      </c>
-      <c r="D156" t="inlineStr">
-        <is>
-          <t>Empyrean</t>
-        </is>
-      </c>
-      <c r="E156" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>69256c61fa804c7cd64e3d0f</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>Lootra</t>
-        </is>
-      </c>
-      <c r="C157" t="n">
-        <v>4</v>
-      </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>Winnu</t>
-        </is>
-      </c>
-      <c r="E157" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>69256c61fa804c7cd64e3d0f</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>Michael 🇦🇹</t>
-        </is>
-      </c>
-      <c r="C158" t="n">
-        <v>3</v>
-      </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t>Saar</t>
-        </is>
-      </c>
-      <c r="E158" t="n">
-        <v>5</v>
-      </c>
-    </row>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add game data: Cleo is onto you, Respect ;-)
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2244,8 +2244,78 @@
       </c>
     </row>
     <row r="46">
-      <c r="D46" s="4" t="n"/>
-      <c r="E46" s="4" t="n"/>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>6a38258dce86419e1a795b30</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Cleo is onto you</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>10</v>
+      </c>
+      <c r="D46" s="4" t="n">
+        <v>46194</v>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>46202</v>
+      </c>
+      <c r="F46" t="n">
+        <v>5</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>1</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>69554f3a40e20c90c204b346</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Respect ;-)</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>10</v>
+      </c>
+      <c r="D47" s="4" t="n">
+        <v>46022</v>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>46195</v>
+      </c>
+      <c r="F47" t="n">
+        <v>7</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Statusphase</t>
+        </is>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2258,7 +2328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E158"/>
+  <dimension ref="A1:E160"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5787,11 +5857,167 @@
         <v>3</v>
       </c>
     </row>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>6a38258dce86419e1a795b30</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Eric</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>9</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Nekro</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>6a38258dce86419e1a795b30</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>10</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Yin</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>6a38258dce86419e1a795b30</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Manu</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>7</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Naalu</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>69554f3a40e20c90c204b346</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Manu</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>9</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Empyrean</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>69554f3a40e20c90c204b346</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Eric</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>8</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Arborec</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>69554f3a40e20c90c204b346</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Fraz</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>8</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Jol</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>69554f3a40e20c90c204b346</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Ketherus</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>10</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Naalu</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove Ketherus game; require core trio (Manu+Thomas+Eric) for group filter
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -2274,6 +2274,9 @@
       <c r="H46" t="n">
         <v>1</v>
       </c>
+      <c r="I46" t="n">
+        <v/>
+      </c>
       <c r="J46" t="inlineStr">
         <is>
           <t>online</t>
@@ -2281,41 +2284,8 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>69554f3a40e20c90c204b346</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Respect ;-)</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>10</v>
-      </c>
-      <c r="D47" s="4" t="n">
-        <v>46022</v>
-      </c>
-      <c r="E47" s="4" t="n">
-        <v>46195</v>
-      </c>
-      <c r="F47" t="n">
-        <v>7</v>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Statusphase</t>
-        </is>
-      </c>
-      <c r="H47" t="n">
-        <v>0</v>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
+      <c r="D47" s="4" t="n"/>
+      <c r="E47" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2328,7 +2298,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E160"/>
+  <dimension ref="A1:E156"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5924,98 +5894,6 @@
       </c>
       <c r="E156" t="n">
         <v>3</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>69554f3a40e20c90c204b346</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>Manu</t>
-        </is>
-      </c>
-      <c r="C157" t="n">
-        <v>9</v>
-      </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>Empyrean</t>
-        </is>
-      </c>
-      <c r="E157" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>69554f3a40e20c90c204b346</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>Eric</t>
-        </is>
-      </c>
-      <c r="C158" t="n">
-        <v>8</v>
-      </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t>Arborec</t>
-        </is>
-      </c>
-      <c r="E158" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>69554f3a40e20c90c204b346</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>Fraz</t>
-        </is>
-      </c>
-      <c r="C159" t="n">
-        <v>8</v>
-      </c>
-      <c r="D159" t="inlineStr">
-        <is>
-          <t>Jol</t>
-        </is>
-      </c>
-      <c r="E159" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>69554f3a40e20c90c204b346</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>Ketherus</t>
-        </is>
-      </c>
-      <c r="C160" t="n">
-        <v>10</v>
-      </c>
-      <c r="D160" t="inlineStr">
-        <is>
-          <t>Naalu</t>
-        </is>
-      </c>
-      <c r="E160" t="n">
-        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add game data: Komm ein schnelles noch
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -2284,8 +2284,41 @@
       </c>
     </row>
     <row r="47">
-      <c r="D47" s="4" t="n"/>
-      <c r="E47" s="4" t="n"/>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>6a436d9c442a0e0c4fbb0567</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Komm ein schnelles noch</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>10</v>
+      </c>
+      <c r="D47" s="4" t="n">
+        <v>46203</v>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>46209</v>
+      </c>
+      <c r="F47" t="n">
+        <v>5</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H47" t="n">
+        <v>1</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2298,7 +2331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E156"/>
+  <dimension ref="A1:E159"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5893,6 +5926,75 @@
         </is>
       </c>
       <c r="E156" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>6a436d9c442a0e0c4fbb0567</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>5</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Mentak</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>6a436d9c442a0e0c4fbb0567</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Manu</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>10</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Yin</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>6a436d9c442a0e0c4fbb0567</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Eric</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>8</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Naalu</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add game data: Diesmal schenke ich Manu aber den Sieg
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2314,7 +2314,47 @@
       <c r="H47" t="n">
         <v>1</v>
       </c>
+      <c r="I47" t="n">
+        <v/>
+      </c>
       <c r="J47" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>6a4b71cec0b6fdb6a6dcfd06</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Diesmal schenke ich Manu aber den Sieg</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>10</v>
+      </c>
+      <c r="D48" s="4" t="n">
+        <v>46209</v>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>46217</v>
+      </c>
+      <c r="F48" t="n">
+        <v>6</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H48" t="n">
+        <v>1</v>
+      </c>
+      <c r="J48" t="inlineStr">
         <is>
           <t>online</t>
         </is>
@@ -2331,7 +2371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E159"/>
+  <dimension ref="A1:E162"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5995,6 +6035,75 @@
         </is>
       </c>
       <c r="E159" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>6a4b71cec0b6fdb6a6dcfd06</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>10</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Winnu</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>6a4b71cec0b6fdb6a6dcfd06</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Eric</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>8</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Saar</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>6a4b71cec0b6fdb6a6dcfd06</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Manu</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>6</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Empyrean</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add game data: SkipToVictory
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2354,7 +2354,47 @@
       <c r="H48" t="n">
         <v>1</v>
       </c>
+      <c r="I48" t="n">
+        <v/>
+      </c>
       <c r="J48" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>6a574898ad0760d27639ab7b</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>SkipToVictory</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>10</v>
+      </c>
+      <c r="D49" s="4" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>46219</v>
+      </c>
+      <c r="F49" t="n">
+        <v>4</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Aktionsphase</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>1</v>
+      </c>
+      <c r="J49" t="inlineStr">
         <is>
           <t>online</t>
         </is>
@@ -2371,7 +2411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E162"/>
+  <dimension ref="A1:E165"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.453125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6104,6 +6144,75 @@
         </is>
       </c>
       <c r="E162" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>6a574898ad0760d27639ab7b</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Eric</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>5</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Xxcha</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>6a574898ad0760d27639ab7b</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>10</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Saar</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>6a574898ad0760d27639ab7b</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Manu</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>3</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Mentak</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>